<commit_message>
export lb and ub
</commit_message>
<xml_diff>
--- a/experiments/results/extended_bound/cplex-cp-extended-bound.xlsx
+++ b/experiments/results/extended_bound/cplex-cp-extended-bound.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,25 +445,35 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Lower bound</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Upper bound</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Best bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Best objective</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -497,25 +507,35 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>26</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>436.0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -545,25 +565,35 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>37</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>9.5</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>5.51</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -597,25 +627,35 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>46</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0.11</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -649,25 +689,35 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>57</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>57</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>20.6</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>45.05</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -701,25 +751,35 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>58</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>58</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>10.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>3.67</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -753,25 +813,35 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>66</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>9.50</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -805,25 +875,35 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>67</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>41.8</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>145.83</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -857,25 +937,35 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>34</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>333.4</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -905,25 +995,35 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>76</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>542.9</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -953,25 +1053,35 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>91</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>116</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>299.8</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1001,25 +1111,35 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>139</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>127.2</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1049,25 +1169,35 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>145</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>145</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>17.1</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>1.14</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1101,25 +1231,35 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>233.4</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>1800.04</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1149,25 +1289,35 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>235.8</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1197,25 +1347,35 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>305</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>429.6</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>1800.03</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1245,25 +1405,35 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>212</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>513</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>308.1</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1293,25 +1463,35 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>570</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>607</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>257.5</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1341,25 +1521,35 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>160</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>604</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>312.9</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1389,25 +1579,35 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>328</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>648</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>265.5</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1437,25 +1637,35 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>264</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>633</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>411.1</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1485,25 +1695,35 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>827</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>827</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>191.7</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>79.05</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1537,25 +1757,35 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>413</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>803</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>386.4</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1585,25 +1815,35 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>325</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>851</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>387.1</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>1800.04</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1633,25 +1873,35 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>286</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>766</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>410.3</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>1800.06</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1664,7 +1914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1695,25 +1945,35 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Lower bound</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Upper bound</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Best bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Best objective</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -1747,25 +2007,35 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>32</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>402.4</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1795,25 +2065,35 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>43</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>43</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>10.9</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>8.81</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1847,25 +2127,35 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>54</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0.09</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1899,25 +2189,35 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>67</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>23.2</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>61.67</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1951,25 +2251,35 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>68</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>6.75</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2003,25 +2313,35 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>78</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>17.97</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2055,25 +2375,35 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>79</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>79</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>55.3</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>242.45</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2107,25 +2437,35 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>37</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>86</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>379.6</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2155,25 +2495,35 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>104</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>118</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>605.6</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2203,25 +2553,35 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>109</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>134</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>285.4</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2251,25 +2611,35 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>154</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>165</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>136.6</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2299,25 +2669,35 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>175</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>175</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>17.8</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>1.15</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2351,25 +2731,35 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>53</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>272.8</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>1800.05</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2399,25 +2789,35 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>53</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>271.7</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2447,25 +2847,35 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>358</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>594</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>548.9</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>1800.04</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2495,25 +2905,35 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>259</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>592</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>437.1</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>1800.04</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2543,25 +2963,35 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>683</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>719</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>224.3</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2591,25 +3021,35 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>190</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>716</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>331.4</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>1800.00</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2639,25 +3079,35 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>393</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>714</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>318.5</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2687,25 +3137,35 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>344</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>717</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>443.3</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>1800.04</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2735,25 +3195,35 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>992</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>992</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>251.2</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>197.93</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2787,25 +3257,35 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>495</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>892</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>419.7</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>1800.02</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2835,25 +3315,35 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>397</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>1021</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>449.7</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>1800.04</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2883,25 +3373,35 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>343</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>908</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>451.4</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>1800.07</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>